<commit_message>
Add separate Übersicht 2025 sheet with monthly income/expense/difference
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFNBQHEzPbML3vXDdVBdxh
</commit_message>
<xml_diff>
--- a/einnahmen/Einnahmen_Ausgaben_2025.xlsx
+++ b/einnahmen/Einnahmen_Ausgaben_2025.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Übersicht 2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2025" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,10 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
     <numFmt numFmtId="165" formatCode="#,##0.00 €;[Red]-#,##0.00 €;-"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="MMMM YYYY"/>
+    <numFmt numFmtId="166" formatCode="MMMM YYYY"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +59,10 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
     </font>
   </fonts>
   <fills count="4">
@@ -108,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,11 +128,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,6 +501,261 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Übersicht 2025 – Einnahmen, Ausgaben, Differenz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Werte aus der Übersicht des Nutzers übernommen (Einnahmen/Ausgaben blau = Eingabe). Ausgaben negativ; Differenz = Einnahmen + Ausgaben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Monat 2025</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Einnahmen (€)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Ausgaben (€)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Differenz (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>-47.28</v>
+      </c>
+      <c r="D5" s="14">
+        <f>B5+C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>-15.9</v>
+      </c>
+      <c r="D6" s="14">
+        <f>B6+C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n">
+        <v>45717</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>-15.9</v>
+      </c>
+      <c r="D7" s="14">
+        <f>B7+C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>-916.3</v>
+      </c>
+      <c r="D8" s="14">
+        <f>B8+C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>-1231.05</v>
+      </c>
+      <c r="D9" s="14">
+        <f>B9+C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>45809</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>-105.96</v>
+      </c>
+      <c r="D10" s="14">
+        <f>B10+C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>-258.77</v>
+      </c>
+      <c r="D11" s="14">
+        <f>B11+C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>600</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>-105.96</v>
+      </c>
+      <c r="D12" s="14">
+        <f>B12+C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>-105.96</v>
+      </c>
+      <c r="D13" s="14">
+        <f>B13+C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>-27.05</v>
+      </c>
+      <c r="D14" s="14">
+        <f>B14+C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>-23.4</v>
+      </c>
+      <c r="D15" s="14">
+        <f>B15+C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>-15.9</v>
+      </c>
+      <c r="D16" s="14">
+        <f>B16+C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Gesamt 2025</t>
+        </is>
+      </c>
+      <c r="B17" s="11">
+        <f>SUM(B5:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="11">
+        <f>SUM(C5:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="11">
+        <f>SUM(D5:D16)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -585,7 +848,7 @@
         <f>IF(A5="","",MONTH(A5))</f>
         <v/>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="15" t="n">
         <v>45658</v>
       </c>
       <c r="I5" s="9">
@@ -611,7 +874,7 @@
         <f>IF(A6="","",MONTH(A6))</f>
         <v/>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="15" t="n">
         <v>45689</v>
       </c>
       <c r="I6" s="9">
@@ -637,7 +900,7 @@
         <f>IF(A7="","",MONTH(A7))</f>
         <v/>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="15" t="n">
         <v>45717</v>
       </c>
       <c r="I7" s="9">
@@ -663,7 +926,7 @@
         <f>IF(A8="","",MONTH(A8))</f>
         <v/>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="15" t="n">
         <v>45748</v>
       </c>
       <c r="I8" s="9">
@@ -689,7 +952,7 @@
         <f>IF(A9="","",MONTH(A9))</f>
         <v/>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="15" t="n">
         <v>45778</v>
       </c>
       <c r="I9" s="9">
@@ -715,7 +978,7 @@
         <f>IF(A10="","",MONTH(A10))</f>
         <v/>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="15" t="n">
         <v>45809</v>
       </c>
       <c r="I10" s="9">
@@ -741,7 +1004,7 @@
         <f>IF(A11="","",MONTH(A11))</f>
         <v/>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="15" t="n">
         <v>45839</v>
       </c>
       <c r="I11" s="9">
@@ -767,7 +1030,7 @@
         <f>IF(A12="","",MONTH(A12))</f>
         <v/>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="15" t="n">
         <v>45870</v>
       </c>
       <c r="I12" s="9">
@@ -793,7 +1056,7 @@
         <f>IF(A13="","",MONTH(A13))</f>
         <v/>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="15" t="n">
         <v>45901</v>
       </c>
       <c r="I13" s="9">
@@ -819,7 +1082,7 @@
         <f>IF(A14="","",MONTH(A14))</f>
         <v/>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="15" t="n">
         <v>45931</v>
       </c>
       <c r="I14" s="9">
@@ -845,7 +1108,7 @@
         <f>IF(A15="","",MONTH(A15))</f>
         <v/>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="15" t="n">
         <v>45962</v>
       </c>
       <c r="I15" s="9">
@@ -871,7 +1134,7 @@
         <f>IF(A16="","",MONTH(A16))</f>
         <v/>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="H16" s="15" t="n">
         <v>45992</v>
       </c>
       <c r="I16" s="9">

</xml_diff>